<commit_message>
Add Railway deployment configuration and documentation
</commit_message>
<xml_diff>
--- a/data/data.xlsx
+++ b/data/data.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="39">
   <si>
     <t>Team Name</t>
   </si>
@@ -104,6 +104,30 @@
   </si>
   <si>
     <t>2025-08-14T08:11:20.607Z</t>
+  </si>
+  <si>
+    <t>T</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>0099009990</t>
+  </si>
+  <si>
+    <t>BE</t>
+  </si>
+  <si>
+    <t>Beginner</t>
+  </si>
+  <si>
+    <t>2025-08-14T12:28:25.965Z</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>2025-08-14T12:34:27.908Z</t>
   </si>
 </sst>
 </file>
@@ -480,7 +504,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:P2"/>
+  <dimension ref="A1:P4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.25">
@@ -583,8 +607,108 @@
         <v>30</v>
       </c>
     </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3" t="s">
+        <v>33</v>
+      </c>
+      <c r="E3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F3" t="s">
+        <v>21</v>
+      </c>
+      <c r="G3" t="s">
+        <v>34</v>
+      </c>
+      <c r="H3" t="s">
+        <v>23</v>
+      </c>
+      <c r="I3" t="s">
+        <v>29</v>
+      </c>
+      <c r="J3" t="s">
+        <v>35</v>
+      </c>
+      <c r="K3" t="s">
+        <v>29</v>
+      </c>
+      <c r="L3" t="s">
+        <v>29</v>
+      </c>
+      <c r="M3" t="s">
+        <v>28</v>
+      </c>
+      <c r="N3" t="s">
+        <v>28</v>
+      </c>
+      <c r="O3" t="s">
+        <v>29</v>
+      </c>
+      <c r="P3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4" t="s">
+        <v>37</v>
+      </c>
+      <c r="C4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D4" t="s">
+        <v>19</v>
+      </c>
+      <c r="E4" t="s">
+        <v>20</v>
+      </c>
+      <c r="F4" t="s">
+        <v>21</v>
+      </c>
+      <c r="G4" t="s">
+        <v>22</v>
+      </c>
+      <c r="H4" t="s">
+        <v>23</v>
+      </c>
+      <c r="I4" t="s">
+        <v>29</v>
+      </c>
+      <c r="J4" t="s">
+        <v>35</v>
+      </c>
+      <c r="K4" t="s">
+        <v>29</v>
+      </c>
+      <c r="L4" t="s">
+        <v>29</v>
+      </c>
+      <c r="M4" t="s">
+        <v>28</v>
+      </c>
+      <c r="N4" t="s">
+        <v>28</v>
+      </c>
+      <c r="O4" t="s">
+        <v>29</v>
+      </c>
+      <c r="P4" t="s">
+        <v>38</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>